<commit_message>
Solve Reassighn Wrong Supplier type
</commit_message>
<xml_diff>
--- a/QuistananirTemplet.xlsx
+++ b/QuistananirTemplet.xlsx
@@ -1,19 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\saed-rpa2\D\FTP\Mivors-Maaden-Edit- CR Registeration request\Mivors-Maaden-Edit- CR Registeration request\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlMufeedM\Documents\UiPath\Live\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF5F2D4F-9298-4DFB-AAA0-A9BA0F9E414E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
   </bookViews>
   <sheets>
-    <sheet name="Quelification" sheetId="2" r:id="rId1"/>
+    <sheet name="Qualification" sheetId="3" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -46,7 +45,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -378,12 +377,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="7" max="7" width="13.81640625" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -409,6 +405,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>